<commit_message>
Update marketing campaign analysis workbook
</commit_message>
<xml_diff>
--- a/excel/marketing_campaign_analysis.xlsx
+++ b/excel/marketing_campaign_analysis.xlsx
@@ -16,6 +16,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Numeric_Audit" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outliers" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Quality_Issue_Log" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleaning_Dictionary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleaning_Summary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Before_After_Categories" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing_Value_Treatment" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Date_Cleaning_Audit" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Currency_Cleaning_Audit" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +30,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -63,11 +71,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,6 +464,911 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>raw_field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>clean_field</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>transformation</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ad_ID</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ad_id</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rename</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Preserve identifier values unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Campaign_Name</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>campaign_name</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rename + standardize</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Map approved campaign variants to Data Analytics Course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>clicks</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rename + numeric conversion</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Convert to numeric; retain missing values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>impressions</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rename + numeric conversion</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Convert to numeric; retain missing values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Rename + currency conversion</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Remove currency symbols/commas and convert to numeric; retain missing values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Leads</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>leads</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Rename + numeric conversion</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Convert to numeric; retain missing values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Conversions</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>conversions</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Rename + numeric conversion</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Convert to numeric; retain missing values; do not infer from Sale_Amount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Conversion Rate</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>conversion_rate</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Rename only</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Retain existing values and missing values. Recalculation deferred to Phase 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sale_Amount</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>sale_amount</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rename + currency conversion</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Remove currency symbols/commas and convert to numeric; retain missing values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ad_Date</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ad_date</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Rename + explicit date parsing</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Parse known YYYY-MM-DD, YYYY/MM/DD and DD-MM-YYYY representations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Rename + standardize</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Map approved Hyderabad variants to Hyderabad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>device</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Rename + case normalization</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Normalize approved device variants to Mobile, Desktop or Tablet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>keyword_raw / keyword_clean</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Preserve + audit field</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Do not arbitrarily merge analytical keyword phrases. Preserve raw values.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cleaned</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2600</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Columns</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C3" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Missing cells</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1150</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Duplicate rows</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Duplicate Ad_ID</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Dimension</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Raw Unique Values</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Cleaned Unique Values</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Campaign</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Device</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>condition</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>record_count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sale_Amount missing</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Conversions missing</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Conversions &gt; 0 and Sale_Amount missing</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sale_Amount &gt; 0 and Conversions missing</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Conversion Rate missing</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Clicks missing</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Impressions missing</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Leads missing</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cost missing</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>97</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Raw date format</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Record count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Parsing format</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Parsing result</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Minimum cleaned date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Maximum cleaned date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NaT count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>893</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>%Y-%m-%d</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>45597</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>45626</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>YYYY/MM/DD</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>844</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>%Y/%m/%d</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>45597</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>45626</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DD-MM-YYYY</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>863</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>%d-%m-%Y</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>45597</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>45626</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Other/unsupported</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Not applicable</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Raw Non-Null Count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Raw Missing Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Cleaned Missing Count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Cleaned Data Type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Remaining Currency Symbols</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Remaining Commas</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Negative Values</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Parsing Failures</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2503</v>
+      </c>
+      <c r="C2" t="n">
+        <v>97</v>
+      </c>
+      <c r="D2" t="n">
+        <v>97</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sale_amount</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2461</v>
+      </c>
+      <c r="C3" t="n">
+        <v>139</v>
+      </c>
+      <c r="D3" t="n">
+        <v>139</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>float64</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1496,8 +2410,6 @@
       <c r="K2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1535,8 +2447,6 @@
       <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1574,8 +2484,6 @@
       <c r="K4" t="n">
         <v>0</v>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1613,8 +2521,6 @@
       <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1649,7 +2555,6 @@
       <c r="J6" t="n">
         <v>0</v>
       </c>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>0</v>
       </c>
@@ -1690,9 +2595,6 @@
       <c r="J7" t="n">
         <v>0</v>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1727,9 +2629,6 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>